<commit_message>
Documentacion y Gantt EA2
</commit_message>
<xml_diff>
--- a/docs/gantt.xlsx
+++ b/docs/gantt.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473D10D0-4049-4A2A-843A-CD3B7A36037E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A851F3E-7F0F-481C-A23A-CF22A61E898C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt" sheetId="11" r:id="rId1"/>
@@ -38,24 +38,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="32">
   <si>
     <t>TAREA</t>
-  </si>
-  <si>
-    <t>Tarea 1</t>
-  </si>
-  <si>
-    <t>Tarea 2</t>
-  </si>
-  <si>
-    <t>Tarea 3</t>
-  </si>
-  <si>
-    <t>Tarea 4</t>
-  </si>
-  <si>
-    <t>Tarea 5</t>
   </si>
   <si>
     <t>Inicio del proyecto:</t>
@@ -120,6 +105,36 @@
   </si>
   <si>
     <t>Etapa 3 – Interpretación y entrega final (EA3)</t>
+  </si>
+  <si>
+    <t>Refinamiento  de Limpieza</t>
+  </si>
+  <si>
+    <t>Enriquecimiento de datos</t>
+  </si>
+  <si>
+    <t>Planeamiento y Desarrollo de Graficas</t>
+  </si>
+  <si>
+    <t>Elaboración Documento APA (Etapa 2)</t>
+  </si>
+  <si>
+    <t>Análisis descriptivo</t>
+  </si>
+  <si>
+    <t>Estructuracion Presentacion</t>
+  </si>
+  <si>
+    <t>Documentacion Proyecto Final</t>
+  </si>
+  <si>
+    <t>Diseño de Dashboard</t>
+  </si>
+  <si>
+    <t>Despliege y Explicacion</t>
+  </si>
+  <si>
+    <t>Presentacion Final</t>
   </si>
 </sst>
 </file>
@@ -1007,23 +1022,23 @@
     <xf numFmtId="14" fontId="7" fillId="8" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="8">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="8" applyBorder="1">
       <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -1591,7 +1606,7 @@
   <sheetData>
     <row r="1" spans="1:62" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="27" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="2"/>
@@ -1602,111 +1617,111 @@
     </row>
     <row r="2" spans="1:62" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="28" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="G2" s="41"/>
     </row>
     <row r="3" spans="1:62" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" s="56" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="57"/>
-      <c r="D3" s="61">
+        <v>20</v>
+      </c>
+      <c r="B3" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="61"/>
+      <c r="D3" s="59">
         <v>45950</v>
       </c>
-      <c r="E3" s="61"/>
+      <c r="E3" s="59"/>
     </row>
     <row r="4" spans="1:62" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="56" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="57"/>
+      <c r="B4" s="60" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="61"/>
       <c r="D4" s="6">
         <v>1</v>
       </c>
-      <c r="G4" s="58">
+      <c r="G4" s="56">
         <f>G5</f>
         <v>45950</v>
       </c>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="59"/>
-      <c r="K4" s="59"/>
-      <c r="L4" s="59"/>
-      <c r="M4" s="60"/>
-      <c r="N4" s="58">
+      <c r="H4" s="57"/>
+      <c r="I4" s="57"/>
+      <c r="J4" s="57"/>
+      <c r="K4" s="57"/>
+      <c r="L4" s="57"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="56">
         <f>N5</f>
         <v>45957</v>
       </c>
-      <c r="O4" s="59"/>
-      <c r="P4" s="59"/>
-      <c r="Q4" s="59"/>
-      <c r="R4" s="59"/>
-      <c r="S4" s="59"/>
-      <c r="T4" s="60"/>
-      <c r="U4" s="58">
+      <c r="O4" s="57"/>
+      <c r="P4" s="57"/>
+      <c r="Q4" s="57"/>
+      <c r="R4" s="57"/>
+      <c r="S4" s="57"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="56">
         <f>U5</f>
         <v>45964</v>
       </c>
-      <c r="V4" s="59"/>
-      <c r="W4" s="59"/>
-      <c r="X4" s="59"/>
-      <c r="Y4" s="59"/>
-      <c r="Z4" s="59"/>
-      <c r="AA4" s="60"/>
-      <c r="AB4" s="58">
+      <c r="V4" s="57"/>
+      <c r="W4" s="57"/>
+      <c r="X4" s="57"/>
+      <c r="Y4" s="57"/>
+      <c r="Z4" s="57"/>
+      <c r="AA4" s="58"/>
+      <c r="AB4" s="56">
         <f>AB5</f>
         <v>45971</v>
       </c>
-      <c r="AC4" s="59"/>
-      <c r="AD4" s="59"/>
-      <c r="AE4" s="59"/>
-      <c r="AF4" s="59"/>
-      <c r="AG4" s="59"/>
-      <c r="AH4" s="60"/>
-      <c r="AI4" s="58">
+      <c r="AC4" s="57"/>
+      <c r="AD4" s="57"/>
+      <c r="AE4" s="57"/>
+      <c r="AF4" s="57"/>
+      <c r="AG4" s="57"/>
+      <c r="AH4" s="58"/>
+      <c r="AI4" s="56">
         <f>AI5</f>
         <v>45978</v>
       </c>
-      <c r="AJ4" s="59"/>
-      <c r="AK4" s="59"/>
-      <c r="AL4" s="59"/>
-      <c r="AM4" s="59"/>
-      <c r="AN4" s="59"/>
-      <c r="AO4" s="60"/>
-      <c r="AP4" s="58">
+      <c r="AJ4" s="57"/>
+      <c r="AK4" s="57"/>
+      <c r="AL4" s="57"/>
+      <c r="AM4" s="57"/>
+      <c r="AN4" s="57"/>
+      <c r="AO4" s="58"/>
+      <c r="AP4" s="56">
         <f>AP5</f>
         <v>45985</v>
       </c>
-      <c r="AQ4" s="59"/>
-      <c r="AR4" s="59"/>
-      <c r="AS4" s="59"/>
-      <c r="AT4" s="59"/>
-      <c r="AU4" s="59"/>
-      <c r="AV4" s="60"/>
-      <c r="AW4" s="58">
+      <c r="AQ4" s="57"/>
+      <c r="AR4" s="57"/>
+      <c r="AS4" s="57"/>
+      <c r="AT4" s="57"/>
+      <c r="AU4" s="57"/>
+      <c r="AV4" s="58"/>
+      <c r="AW4" s="56">
         <f>AW5</f>
         <v>45992</v>
       </c>
-      <c r="AX4" s="59"/>
-      <c r="AY4" s="59"/>
-      <c r="AZ4" s="59"/>
-      <c r="BA4" s="59"/>
-      <c r="BB4" s="59"/>
-      <c r="BC4" s="60"/>
-      <c r="BD4" s="58">
+      <c r="AX4" s="57"/>
+      <c r="AY4" s="57"/>
+      <c r="AZ4" s="57"/>
+      <c r="BA4" s="57"/>
+      <c r="BB4" s="57"/>
+      <c r="BC4" s="58"/>
+      <c r="BD4" s="56">
         <f>BD5</f>
         <v>45999</v>
       </c>
-      <c r="BE4" s="59"/>
-      <c r="BF4" s="59"/>
-      <c r="BG4" s="59"/>
-      <c r="BH4" s="59"/>
-      <c r="BI4" s="59"/>
-      <c r="BJ4" s="60"/>
+      <c r="BE4" s="57"/>
+      <c r="BF4" s="57"/>
+      <c r="BG4" s="57"/>
+      <c r="BH4" s="57"/>
+      <c r="BI4" s="57"/>
+      <c r="BJ4" s="58"/>
     </row>
     <row r="5" spans="1:62" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="39"/>
@@ -1944,19 +1959,19 @@
         <v>0</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D6" s="46" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E6" s="46" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="G6" s="9" t="str">
         <f t="shared" ref="G6" si="3">LEFT(TEXT(G5,"ddd"),1)</f>
@@ -2250,7 +2265,7 @@
     </row>
     <row r="8" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B8" s="30"/>
       <c r="C8" s="14">
@@ -2325,10 +2340,10 @@
     </row>
     <row r="9" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="36" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B9" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C9" s="15">
         <v>1</v>
@@ -2404,10 +2419,10 @@
     </row>
     <row r="10" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="36" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B10" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C10" s="15">
         <v>1</v>
@@ -2481,10 +2496,10 @@
     </row>
     <row r="11" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="36" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B11" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C11" s="15">
         <v>1</v>
@@ -2558,10 +2573,10 @@
     </row>
     <row r="12" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="36" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B12" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C12" s="15">
         <v>1</v>
@@ -2635,10 +2650,10 @@
     </row>
     <row r="13" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="36" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B13" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C13" s="15">
         <v>1</v>
@@ -2712,10 +2727,10 @@
     </row>
     <row r="14" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B14" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C14" s="15">
         <v>1</v>
@@ -2789,10 +2804,10 @@
     </row>
     <row r="15" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="36" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B15" s="31" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C15" s="15">
         <v>1</v>
@@ -2866,11 +2881,11 @@
     </row>
     <row r="16" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B16" s="32"/>
       <c r="C16" s="17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="50">
         <v>45971</v>
@@ -2941,23 +2956,23 @@
     </row>
     <row r="17" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="18">
         <v>1</v>
       </c>
-      <c r="B17" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="18">
-        <v>0</v>
-      </c>
       <c r="D17" s="52">
-        <v>45971</v>
+        <v>45978</v>
       </c>
       <c r="E17" s="52">
-        <v>45984</v>
+        <v>45979</v>
       </c>
       <c r="F17" s="12">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G17" s="22"/>
       <c r="H17" s="22"/>
@@ -3018,23 +3033,23 @@
     </row>
     <row r="18" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="37" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B18" s="33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C18" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="52">
-        <v>45971</v>
+        <v>45980</v>
       </c>
       <c r="E18" s="52">
-        <v>45984</v>
+        <v>45982</v>
       </c>
       <c r="F18" s="12">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="G18" s="22"/>
       <c r="H18" s="22"/>
@@ -3095,23 +3110,23 @@
     </row>
     <row r="19" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="37" t="s">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="B19" s="33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C19" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D19" s="52">
-        <v>45971</v>
+        <v>45983</v>
       </c>
       <c r="E19" s="52">
-        <v>45984</v>
+        <v>45983</v>
       </c>
       <c r="F19" s="12">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G19" s="22"/>
       <c r="H19" s="22"/>
@@ -3172,23 +3187,23 @@
     </row>
     <row r="20" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="37" t="s">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C20" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" s="52">
-        <v>45971</v>
+        <v>45984</v>
       </c>
       <c r="E20" s="52">
         <v>45984</v>
       </c>
       <c r="F20" s="12">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G20" s="22"/>
       <c r="H20" s="22"/>
@@ -3249,23 +3264,23 @@
     </row>
     <row r="21" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="37" t="s">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B21" s="33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C21" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D21" s="52">
-        <v>45971</v>
+        <v>45984</v>
       </c>
       <c r="E21" s="52">
         <v>45984</v>
       </c>
       <c r="F21" s="12">
         <f t="shared" si="6"/>
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="G21" s="22"/>
       <c r="H21" s="22"/>
@@ -3326,7 +3341,7 @@
     </row>
     <row r="22" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B22" s="34"/>
       <c r="C22" s="20">
@@ -3401,10 +3416,10 @@
     </row>
     <row r="23" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="38" t="s">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="B23" s="35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C23" s="21">
         <v>0</v>
@@ -3478,10 +3493,10 @@
     </row>
     <row r="24" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="38" t="s">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="B24" s="35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C24" s="21">
         <v>0</v>
@@ -3555,10 +3570,10 @@
     </row>
     <row r="25" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="38" t="s">
-        <v>3</v>
+        <v>29</v>
       </c>
       <c r="B25" s="35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C25" s="21">
         <v>0</v>
@@ -3632,10 +3647,10 @@
     </row>
     <row r="26" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="38" t="s">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="B26" s="35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C26" s="21">
         <v>0</v>
@@ -3709,10 +3724,10 @@
     </row>
     <row r="27" spans="1:62" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="38" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B27" s="35" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C27" s="21">
         <v>0</v>
@@ -3793,17 +3808,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="AI4:AO4"/>
+    <mergeCell ref="AP4:AV4"/>
+    <mergeCell ref="AW4:BC4"/>
     <mergeCell ref="BD4:BJ4"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="G4:M4"/>
     <mergeCell ref="N4:T4"/>
     <mergeCell ref="U4:AA4"/>
     <mergeCell ref="AB4:AH4"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="AI4:AO4"/>
-    <mergeCell ref="AP4:AV4"/>
-    <mergeCell ref="AW4:BC4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C27">
     <cfRule type="dataBar" priority="14">
@@ -4156,15 +4171,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -4182,6 +4188,15 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4206,14 +4221,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -4223,4 +4230,12 @@
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>